<commit_message>
Add sites placeholder in all reports
</commit_message>
<xml_diff>
--- a/api/templates/inventory_log/en.xlsx
+++ b/api/templates/inventory_log/en.xlsx
@@ -1,140 +1,139 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\inventory_log\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="815"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Inventory Log" sheetId="2" r:id="rId1"/>
+    <sheet name="Inventory Log" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913" fullPrecision="0"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <extLst>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
-    <t>&lt;Table&gt;</t>
+    <t xml:space="preserve">Inventory Log</t>
   </si>
   <si>
-    <t>Dates: &lt;Dates&gt;</t>
+    <t xml:space="preserve">Dates: &lt;Dates&gt;</t>
   </si>
   <si>
-    <t>Inventory Log</t>
+    <t xml:space="preserve">&lt;StatesLabel&gt;: &lt;States&gt;</t>
   </si>
   <si>
-    <t>Date</t>
+    <t xml:space="preserve">&lt;LgasLabel&gt;: &lt;Lgas&gt;</t>
   </si>
   <si>
-    <t>Consumable</t>
+    <t xml:space="preserve">&lt;SitesLabel&gt;: &lt;Sites&gt;</t>
   </si>
   <si>
-    <t>Lot</t>
+    <t xml:space="preserve">&lt;Table&gt;</t>
   </si>
   <si>
-    <t>Expiration Date</t>
+    <t xml:space="preserve">Date</t>
   </si>
   <si>
-    <t>Site</t>
+    <t xml:space="preserve">Consumable</t>
   </si>
   <si>
-    <t>Reason</t>
+    <t xml:space="preserve">Lot</t>
   </si>
   <si>
-    <t>Quantity</t>
+    <t xml:space="preserve">Expiration Date</t>
   </si>
   <si>
-    <t>&lt;consumableName&gt;</t>
+    <t xml:space="preserve">Site</t>
   </si>
   <si>
-    <t>&lt;lotNumber&gt;</t>
+    <t xml:space="preserve">Reason</t>
   </si>
   <si>
-    <t>&lt;expirationDate&gt;</t>
+    <t xml:space="preserve">Quantity</t>
   </si>
   <si>
-    <t>&lt;siteName&gt;</t>
+    <t xml:space="preserve">Notes</t>
   </si>
   <si>
-    <t>&lt;movementReason&gt;</t>
+    <t xml:space="preserve">&lt;createdOn&gt;</t>
   </si>
   <si>
-    <t>&lt;quantity&gt;</t>
+    <t xml:space="preserve">&lt;consumableName&gt;</t>
   </si>
   <si>
-    <t>Notes</t>
+    <t xml:space="preserve">&lt;lotNumber&gt;</t>
   </si>
   <si>
-    <t>&lt;notes&gt;</t>
+    <t xml:space="preserve">&lt;expirationDate&gt;</t>
   </si>
   <si>
-    <t>&lt;createdOn&gt;</t>
+    <t xml:space="preserve">&lt;siteName&gt;</t>
   </si>
   <si>
-    <t>&lt;StatesLabel&gt;: &lt;States&gt;</t>
+    <t xml:space="preserve">&lt;movementReason&gt;</t>
   </si>
   <si>
-    <t>&lt;LgasLabel&gt;: &lt;Lgas&gt;</t>
+    <t xml:space="preserve">&lt;quantity&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;notes&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+    <numFmt numFmtId="166" formatCode="0%"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="12"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="16"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
     </font>
     <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <b val="true"/>
       <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -147,514 +146,184 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF3CC0DD"/>
+        <bgColor rgb="FF00CCFF"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="2">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="44">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="43" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="10">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="44">
-    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="43" builtinId="5"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD7D7D7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
-  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
-      <tableStyleElement type="wholeTable" dxfId="1"/>
-      <tableStyleElement type="headerRow" dxfId="0"/>
-    </tableStyle>
-  </tableStyles>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF3CC0DD"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H335"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H336"/>
+  <sheetFormatPr defaultColWidth="11.21484375" defaultRowHeight="15.6" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="20.8984375" style="8" customWidth="1"/>
-    <col min="2" max="2" width="33" customWidth="1"/>
-    <col min="3" max="3" width="14.69921875" customWidth="1"/>
-    <col min="4" max="4" width="19.796875" customWidth="1"/>
-    <col min="5" max="5" width="30.5" customWidth="1"/>
-    <col min="6" max="6" width="28.19921875" customWidth="1"/>
-    <col min="8" max="8" width="56.296875" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="28.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="56.3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="4" t="s">
-        <v>2</v>
+    <row r="1" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -662,7 +331,7 @@
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -672,9 +341,9 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -682,9 +351,9 @@
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -692,2367 +361,2382 @@
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="3"/>
+    <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="1:8" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>0</v>
-      </c>
+    <row r="6" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:8" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="5" t="s">
+    <row r="7" customFormat="false" ht="16.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="16.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="E8" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="D9" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>10</v>
+      <c r="F9" s="9" t="s">
+        <v>19</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>11</v>
+      <c r="G9" s="9" t="s">
+        <v>20</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>12</v>
+      <c r="H9" s="9" t="s">
+        <v>21</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="17" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="18" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="19" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="31" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="32" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="33" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="34" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="35" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="36" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="37" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="38" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="39" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="40" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="41" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="42" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="43" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="44" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="45" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="46" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="47" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="48" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="49" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="50" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="51" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="52" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="53" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="54" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="55" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="56" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="57" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="58" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="59" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="60" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="61" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="62" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="63" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="64" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="65" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="66" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
       <c r="D66" s="3"/>
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="67" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
       <c r="D67" s="3"/>
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="68" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
       <c r="D68" s="3"/>
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="69" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
       <c r="D69" s="3"/>
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="70" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
       <c r="D70" s="3"/>
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="71" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
       <c r="D71" s="3"/>
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="72" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
       <c r="D72" s="3"/>
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="73" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
       <c r="D73" s="3"/>
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="74" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="D74" s="3"/>
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="75" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
       <c r="D75" s="3"/>
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="76" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="77" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="78" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="79" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="80" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="81" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="82" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="83" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="84" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="85" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="86" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="87" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="88" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="89" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="90" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="91" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="92" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="93" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="94" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="95" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="96" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="97" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="98" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="99" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="100" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="101" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>
       <c r="E101" s="3"/>
       <c r="F101" s="3"/>
     </row>
-    <row r="102" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="102" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
       <c r="D102" s="3"/>
       <c r="E102" s="3"/>
       <c r="F102" s="3"/>
     </row>
-    <row r="103" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="103" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
       <c r="D103" s="3"/>
       <c r="E103" s="3"/>
       <c r="F103" s="3"/>
     </row>
-    <row r="104" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="104" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
       <c r="D104" s="3"/>
       <c r="E104" s="3"/>
       <c r="F104" s="3"/>
     </row>
-    <row r="105" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="105" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
       <c r="D105" s="3"/>
       <c r="E105" s="3"/>
       <c r="F105" s="3"/>
     </row>
-    <row r="106" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="106" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
       <c r="F106" s="3"/>
     </row>
-    <row r="107" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="107" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
       <c r="D107" s="3"/>
       <c r="E107" s="3"/>
       <c r="F107" s="3"/>
     </row>
-    <row r="108" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="108" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
       <c r="E108" s="3"/>
       <c r="F108" s="3"/>
     </row>
-    <row r="109" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="109" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
       <c r="D109" s="3"/>
       <c r="E109" s="3"/>
       <c r="F109" s="3"/>
     </row>
-    <row r="110" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="110" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
       <c r="D110" s="3"/>
       <c r="E110" s="3"/>
       <c r="F110" s="3"/>
     </row>
-    <row r="111" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="111" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
       <c r="D111" s="3"/>
       <c r="E111" s="3"/>
       <c r="F111" s="3"/>
     </row>
-    <row r="112" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="112" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
       <c r="D112" s="3"/>
       <c r="E112" s="3"/>
       <c r="F112" s="3"/>
     </row>
-    <row r="113" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="113" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
       <c r="D113" s="3"/>
       <c r="E113" s="3"/>
       <c r="F113" s="3"/>
     </row>
-    <row r="114" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="114" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
       <c r="D114" s="3"/>
       <c r="E114" s="3"/>
       <c r="F114" s="3"/>
     </row>
-    <row r="115" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="115" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
       <c r="D115" s="3"/>
       <c r="E115" s="3"/>
       <c r="F115" s="3"/>
     </row>
-    <row r="116" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="116" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
       <c r="D116" s="3"/>
       <c r="E116" s="3"/>
       <c r="F116" s="3"/>
     </row>
-    <row r="117" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="117" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
       <c r="D117" s="3"/>
       <c r="E117" s="3"/>
       <c r="F117" s="3"/>
     </row>
-    <row r="118" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="118" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
       <c r="D118" s="3"/>
       <c r="E118" s="3"/>
       <c r="F118" s="3"/>
     </row>
-    <row r="119" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="119" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
       <c r="D119" s="3"/>
       <c r="E119" s="3"/>
       <c r="F119" s="3"/>
     </row>
-    <row r="120" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="120" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
       <c r="D120" s="3"/>
       <c r="E120" s="3"/>
       <c r="F120" s="3"/>
     </row>
-    <row r="121" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="121" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
       <c r="D121" s="3"/>
       <c r="E121" s="3"/>
       <c r="F121" s="3"/>
     </row>
-    <row r="122" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="122" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
       <c r="D122" s="3"/>
       <c r="E122" s="3"/>
       <c r="F122" s="3"/>
     </row>
-    <row r="123" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="123" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
       <c r="D123" s="3"/>
       <c r="E123" s="3"/>
       <c r="F123" s="3"/>
     </row>
-    <row r="124" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="124" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
       <c r="D124" s="3"/>
       <c r="E124" s="3"/>
       <c r="F124" s="3"/>
     </row>
-    <row r="125" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="125" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
       <c r="D125" s="3"/>
       <c r="E125" s="3"/>
       <c r="F125" s="3"/>
     </row>
-    <row r="126" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="126" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
       <c r="D126" s="3"/>
       <c r="E126" s="3"/>
       <c r="F126" s="3"/>
     </row>
-    <row r="127" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="127" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
       <c r="D127" s="3"/>
       <c r="E127" s="3"/>
       <c r="F127" s="3"/>
     </row>
-    <row r="128" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="128" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
       <c r="D128" s="3"/>
       <c r="E128" s="3"/>
       <c r="F128" s="3"/>
     </row>
-    <row r="129" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="129" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
       <c r="D129" s="3"/>
       <c r="E129" s="3"/>
       <c r="F129" s="3"/>
     </row>
-    <row r="130" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="130" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
       <c r="D130" s="3"/>
       <c r="E130" s="3"/>
       <c r="F130" s="3"/>
     </row>
-    <row r="131" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="131" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
       <c r="D131" s="3"/>
       <c r="E131" s="3"/>
       <c r="F131" s="3"/>
     </row>
-    <row r="132" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="132" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
       <c r="D132" s="3"/>
       <c r="E132" s="3"/>
       <c r="F132" s="3"/>
     </row>
-    <row r="133" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="133" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
       <c r="D133" s="3"/>
       <c r="E133" s="3"/>
       <c r="F133" s="3"/>
     </row>
-    <row r="134" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="134" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
       <c r="D134" s="3"/>
       <c r="E134" s="3"/>
       <c r="F134" s="3"/>
     </row>
-    <row r="135" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="135" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
       <c r="D135" s="3"/>
       <c r="E135" s="3"/>
       <c r="F135" s="3"/>
     </row>
-    <row r="136" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="136" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
       <c r="D136" s="3"/>
       <c r="E136" s="3"/>
       <c r="F136" s="3"/>
     </row>
-    <row r="137" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="137" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B137" s="3"/>
       <c r="C137" s="3"/>
       <c r="D137" s="3"/>
       <c r="E137" s="3"/>
       <c r="F137" s="3"/>
     </row>
-    <row r="138" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="138" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B138" s="3"/>
       <c r="C138" s="3"/>
       <c r="D138" s="3"/>
       <c r="E138" s="3"/>
       <c r="F138" s="3"/>
     </row>
-    <row r="139" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="139" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
       <c r="D139" s="3"/>
       <c r="E139" s="3"/>
       <c r="F139" s="3"/>
     </row>
-    <row r="140" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="140" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
       <c r="D140" s="3"/>
       <c r="E140" s="3"/>
       <c r="F140" s="3"/>
     </row>
-    <row r="141" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="141" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
       <c r="D141" s="3"/>
       <c r="E141" s="3"/>
       <c r="F141" s="3"/>
     </row>
-    <row r="142" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="142" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
       <c r="D142" s="3"/>
       <c r="E142" s="3"/>
       <c r="F142" s="3"/>
     </row>
-    <row r="143" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="143" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
       <c r="D143" s="3"/>
       <c r="E143" s="3"/>
       <c r="F143" s="3"/>
     </row>
-    <row r="144" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="144" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>
       <c r="D144" s="3"/>
       <c r="E144" s="3"/>
       <c r="F144" s="3"/>
     </row>
-    <row r="145" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="145" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B145" s="3"/>
       <c r="C145" s="3"/>
       <c r="D145" s="3"/>
       <c r="E145" s="3"/>
       <c r="F145" s="3"/>
     </row>
-    <row r="146" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="146" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
       <c r="D146" s="3"/>
       <c r="E146" s="3"/>
       <c r="F146" s="3"/>
     </row>
-    <row r="147" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="147" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
       <c r="D147" s="3"/>
       <c r="E147" s="3"/>
       <c r="F147" s="3"/>
     </row>
-    <row r="148" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="148" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
       <c r="D148" s="3"/>
       <c r="E148" s="3"/>
       <c r="F148" s="3"/>
     </row>
-    <row r="149" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="149" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B149" s="3"/>
       <c r="C149" s="3"/>
       <c r="D149" s="3"/>
       <c r="E149" s="3"/>
       <c r="F149" s="3"/>
     </row>
-    <row r="150" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="150" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B150" s="3"/>
       <c r="C150" s="3"/>
       <c r="D150" s="3"/>
       <c r="E150" s="3"/>
       <c r="F150" s="3"/>
     </row>
-    <row r="151" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="151" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B151" s="3"/>
       <c r="C151" s="3"/>
       <c r="D151" s="3"/>
       <c r="E151" s="3"/>
       <c r="F151" s="3"/>
     </row>
-    <row r="152" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="152" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B152" s="3"/>
       <c r="C152" s="3"/>
       <c r="D152" s="3"/>
       <c r="E152" s="3"/>
       <c r="F152" s="3"/>
     </row>
-    <row r="153" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="153" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B153" s="3"/>
       <c r="C153" s="3"/>
       <c r="D153" s="3"/>
       <c r="E153" s="3"/>
       <c r="F153" s="3"/>
     </row>
-    <row r="154" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="154" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B154" s="3"/>
       <c r="C154" s="3"/>
       <c r="D154" s="3"/>
       <c r="E154" s="3"/>
       <c r="F154" s="3"/>
     </row>
-    <row r="155" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="155" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B155" s="3"/>
       <c r="C155" s="3"/>
       <c r="D155" s="3"/>
       <c r="E155" s="3"/>
       <c r="F155" s="3"/>
     </row>
-    <row r="156" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="156" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B156" s="3"/>
       <c r="C156" s="3"/>
       <c r="D156" s="3"/>
       <c r="E156" s="3"/>
       <c r="F156" s="3"/>
     </row>
-    <row r="157" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="157" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B157" s="3"/>
       <c r="C157" s="3"/>
       <c r="D157" s="3"/>
       <c r="E157" s="3"/>
       <c r="F157" s="3"/>
     </row>
-    <row r="158" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="158" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="3"/>
       <c r="C158" s="3"/>
       <c r="D158" s="3"/>
       <c r="E158" s="3"/>
       <c r="F158" s="3"/>
     </row>
-    <row r="159" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="159" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B159" s="3"/>
       <c r="C159" s="3"/>
       <c r="D159" s="3"/>
       <c r="E159" s="3"/>
       <c r="F159" s="3"/>
     </row>
-    <row r="160" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="160" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B160" s="3"/>
       <c r="C160" s="3"/>
       <c r="D160" s="3"/>
       <c r="E160" s="3"/>
       <c r="F160" s="3"/>
     </row>
-    <row r="161" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="161" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B161" s="3"/>
       <c r="C161" s="3"/>
       <c r="D161" s="3"/>
       <c r="E161" s="3"/>
       <c r="F161" s="3"/>
     </row>
-    <row r="162" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="162" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B162" s="3"/>
       <c r="C162" s="3"/>
       <c r="D162" s="3"/>
       <c r="E162" s="3"/>
       <c r="F162" s="3"/>
     </row>
-    <row r="163" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="163" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B163" s="3"/>
       <c r="C163" s="3"/>
       <c r="D163" s="3"/>
       <c r="E163" s="3"/>
       <c r="F163" s="3"/>
     </row>
-    <row r="164" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="164" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B164" s="3"/>
       <c r="C164" s="3"/>
       <c r="D164" s="3"/>
       <c r="E164" s="3"/>
       <c r="F164" s="3"/>
     </row>
-    <row r="165" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="165" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B165" s="3"/>
       <c r="C165" s="3"/>
       <c r="D165" s="3"/>
       <c r="E165" s="3"/>
       <c r="F165" s="3"/>
     </row>
-    <row r="166" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="166" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="3"/>
       <c r="C166" s="3"/>
       <c r="D166" s="3"/>
       <c r="E166" s="3"/>
       <c r="F166" s="3"/>
     </row>
-    <row r="167" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="167" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B167" s="3"/>
       <c r="C167" s="3"/>
       <c r="D167" s="3"/>
       <c r="E167" s="3"/>
       <c r="F167" s="3"/>
     </row>
-    <row r="168" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="168" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="3"/>
       <c r="C168" s="3"/>
       <c r="D168" s="3"/>
       <c r="E168" s="3"/>
       <c r="F168" s="3"/>
     </row>
-    <row r="169" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="169" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="3"/>
       <c r="C169" s="3"/>
       <c r="D169" s="3"/>
       <c r="E169" s="3"/>
       <c r="F169" s="3"/>
     </row>
-    <row r="170" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="170" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B170" s="3"/>
       <c r="C170" s="3"/>
       <c r="D170" s="3"/>
       <c r="E170" s="3"/>
       <c r="F170" s="3"/>
     </row>
-    <row r="171" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="171" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B171" s="3"/>
       <c r="C171" s="3"/>
       <c r="D171" s="3"/>
       <c r="E171" s="3"/>
       <c r="F171" s="3"/>
     </row>
-    <row r="172" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="172" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B172" s="3"/>
       <c r="C172" s="3"/>
       <c r="D172" s="3"/>
       <c r="E172" s="3"/>
       <c r="F172" s="3"/>
     </row>
-    <row r="173" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="173" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B173" s="3"/>
       <c r="C173" s="3"/>
       <c r="D173" s="3"/>
       <c r="E173" s="3"/>
       <c r="F173" s="3"/>
     </row>
-    <row r="174" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="174" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B174" s="3"/>
       <c r="C174" s="3"/>
       <c r="D174" s="3"/>
       <c r="E174" s="3"/>
       <c r="F174" s="3"/>
     </row>
-    <row r="175" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="175" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B175" s="3"/>
       <c r="C175" s="3"/>
       <c r="D175" s="3"/>
       <c r="E175" s="3"/>
       <c r="F175" s="3"/>
     </row>
-    <row r="176" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="176" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B176" s="3"/>
       <c r="C176" s="3"/>
       <c r="D176" s="3"/>
       <c r="E176" s="3"/>
       <c r="F176" s="3"/>
     </row>
-    <row r="177" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="177" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B177" s="3"/>
       <c r="C177" s="3"/>
       <c r="D177" s="3"/>
       <c r="E177" s="3"/>
       <c r="F177" s="3"/>
     </row>
-    <row r="178" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="178" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B178" s="3"/>
       <c r="C178" s="3"/>
       <c r="D178" s="3"/>
       <c r="E178" s="3"/>
       <c r="F178" s="3"/>
     </row>
-    <row r="179" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="179" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B179" s="3"/>
       <c r="C179" s="3"/>
       <c r="D179" s="3"/>
       <c r="E179" s="3"/>
       <c r="F179" s="3"/>
     </row>
-    <row r="180" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="180" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B180" s="3"/>
       <c r="C180" s="3"/>
       <c r="D180" s="3"/>
       <c r="E180" s="3"/>
       <c r="F180" s="3"/>
     </row>
-    <row r="181" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="181" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B181" s="3"/>
       <c r="C181" s="3"/>
       <c r="D181" s="3"/>
       <c r="E181" s="3"/>
       <c r="F181" s="3"/>
     </row>
-    <row r="182" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="182" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B182" s="3"/>
       <c r="C182" s="3"/>
       <c r="D182" s="3"/>
       <c r="E182" s="3"/>
       <c r="F182" s="3"/>
     </row>
-    <row r="183" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="183" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B183" s="3"/>
       <c r="C183" s="3"/>
       <c r="D183" s="3"/>
       <c r="E183" s="3"/>
       <c r="F183" s="3"/>
     </row>
-    <row r="184" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="184" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B184" s="3"/>
       <c r="C184" s="3"/>
       <c r="D184" s="3"/>
       <c r="E184" s="3"/>
       <c r="F184" s="3"/>
     </row>
-    <row r="185" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="185" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B185" s="3"/>
       <c r="C185" s="3"/>
       <c r="D185" s="3"/>
       <c r="E185" s="3"/>
       <c r="F185" s="3"/>
     </row>
-    <row r="186" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="186" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B186" s="3"/>
       <c r="C186" s="3"/>
       <c r="D186" s="3"/>
       <c r="E186" s="3"/>
       <c r="F186" s="3"/>
     </row>
-    <row r="187" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="187" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B187" s="3"/>
       <c r="C187" s="3"/>
       <c r="D187" s="3"/>
       <c r="E187" s="3"/>
       <c r="F187" s="3"/>
     </row>
-    <row r="188" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="188" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B188" s="3"/>
       <c r="C188" s="3"/>
       <c r="D188" s="3"/>
       <c r="E188" s="3"/>
       <c r="F188" s="3"/>
     </row>
-    <row r="189" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="189" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B189" s="3"/>
       <c r="C189" s="3"/>
       <c r="D189" s="3"/>
       <c r="E189" s="3"/>
       <c r="F189" s="3"/>
     </row>
-    <row r="190" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="190" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B190" s="3"/>
       <c r="C190" s="3"/>
       <c r="D190" s="3"/>
       <c r="E190" s="3"/>
       <c r="F190" s="3"/>
     </row>
-    <row r="191" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="191" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B191" s="3"/>
       <c r="C191" s="3"/>
       <c r="D191" s="3"/>
       <c r="E191" s="3"/>
       <c r="F191" s="3"/>
     </row>
-    <row r="192" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="192" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B192" s="3"/>
       <c r="C192" s="3"/>
       <c r="D192" s="3"/>
       <c r="E192" s="3"/>
       <c r="F192" s="3"/>
     </row>
-    <row r="193" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="193" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B193" s="3"/>
       <c r="C193" s="3"/>
       <c r="D193" s="3"/>
       <c r="E193" s="3"/>
       <c r="F193" s="3"/>
     </row>
-    <row r="194" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="194" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B194" s="3"/>
       <c r="C194" s="3"/>
       <c r="D194" s="3"/>
       <c r="E194" s="3"/>
       <c r="F194" s="3"/>
     </row>
-    <row r="195" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="195" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B195" s="3"/>
       <c r="C195" s="3"/>
       <c r="D195" s="3"/>
       <c r="E195" s="3"/>
       <c r="F195" s="3"/>
     </row>
-    <row r="196" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="196" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B196" s="3"/>
       <c r="C196" s="3"/>
       <c r="D196" s="3"/>
       <c r="E196" s="3"/>
       <c r="F196" s="3"/>
     </row>
-    <row r="197" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="197" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B197" s="3"/>
       <c r="C197" s="3"/>
       <c r="D197" s="3"/>
       <c r="E197" s="3"/>
       <c r="F197" s="3"/>
     </row>
-    <row r="198" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="198" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B198" s="3"/>
       <c r="C198" s="3"/>
       <c r="D198" s="3"/>
       <c r="E198" s="3"/>
       <c r="F198" s="3"/>
     </row>
-    <row r="199" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="199" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B199" s="3"/>
       <c r="C199" s="3"/>
       <c r="D199" s="3"/>
       <c r="E199" s="3"/>
       <c r="F199" s="3"/>
     </row>
-    <row r="200" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="200" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B200" s="3"/>
       <c r="C200" s="3"/>
       <c r="D200" s="3"/>
       <c r="E200" s="3"/>
       <c r="F200" s="3"/>
     </row>
-    <row r="201" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="201" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B201" s="3"/>
       <c r="C201" s="3"/>
       <c r="D201" s="3"/>
       <c r="E201" s="3"/>
       <c r="F201" s="3"/>
     </row>
-    <row r="202" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="202" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B202" s="3"/>
       <c r="C202" s="3"/>
       <c r="D202" s="3"/>
       <c r="E202" s="3"/>
       <c r="F202" s="3"/>
     </row>
-    <row r="203" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="203" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B203" s="3"/>
       <c r="C203" s="3"/>
       <c r="D203" s="3"/>
       <c r="E203" s="3"/>
       <c r="F203" s="3"/>
     </row>
-    <row r="204" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="204" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B204" s="3"/>
       <c r="C204" s="3"/>
       <c r="D204" s="3"/>
       <c r="E204" s="3"/>
       <c r="F204" s="3"/>
     </row>
-    <row r="205" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="205" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B205" s="3"/>
       <c r="C205" s="3"/>
       <c r="D205" s="3"/>
       <c r="E205" s="3"/>
       <c r="F205" s="3"/>
     </row>
-    <row r="206" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="206" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B206" s="3"/>
       <c r="C206" s="3"/>
       <c r="D206" s="3"/>
       <c r="E206" s="3"/>
       <c r="F206" s="3"/>
     </row>
-    <row r="207" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="207" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B207" s="3"/>
       <c r="C207" s="3"/>
       <c r="D207" s="3"/>
       <c r="E207" s="3"/>
       <c r="F207" s="3"/>
     </row>
-    <row r="208" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="208" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B208" s="3"/>
       <c r="C208" s="3"/>
       <c r="D208" s="3"/>
       <c r="E208" s="3"/>
       <c r="F208" s="3"/>
     </row>
-    <row r="209" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="209" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B209" s="3"/>
       <c r="C209" s="3"/>
       <c r="D209" s="3"/>
       <c r="E209" s="3"/>
       <c r="F209" s="3"/>
     </row>
-    <row r="210" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="210" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B210" s="3"/>
       <c r="C210" s="3"/>
       <c r="D210" s="3"/>
       <c r="E210" s="3"/>
       <c r="F210" s="3"/>
     </row>
-    <row r="211" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="211" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B211" s="3"/>
       <c r="C211" s="3"/>
       <c r="D211" s="3"/>
       <c r="E211" s="3"/>
       <c r="F211" s="3"/>
     </row>
-    <row r="212" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="212" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B212" s="3"/>
       <c r="C212" s="3"/>
       <c r="D212" s="3"/>
       <c r="E212" s="3"/>
       <c r="F212" s="3"/>
     </row>
-    <row r="213" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="213" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B213" s="3"/>
       <c r="C213" s="3"/>
       <c r="D213" s="3"/>
       <c r="E213" s="3"/>
       <c r="F213" s="3"/>
     </row>
-    <row r="214" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="214" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B214" s="3"/>
       <c r="C214" s="3"/>
       <c r="D214" s="3"/>
       <c r="E214" s="3"/>
       <c r="F214" s="3"/>
     </row>
-    <row r="215" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="215" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B215" s="3"/>
       <c r="C215" s="3"/>
       <c r="D215" s="3"/>
       <c r="E215" s="3"/>
       <c r="F215" s="3"/>
     </row>
-    <row r="216" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="216" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B216" s="3"/>
       <c r="C216" s="3"/>
       <c r="D216" s="3"/>
       <c r="E216" s="3"/>
       <c r="F216" s="3"/>
     </row>
-    <row r="217" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="217" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B217" s="3"/>
       <c r="C217" s="3"/>
       <c r="D217" s="3"/>
       <c r="E217" s="3"/>
       <c r="F217" s="3"/>
     </row>
-    <row r="218" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="218" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B218" s="3"/>
       <c r="C218" s="3"/>
       <c r="D218" s="3"/>
       <c r="E218" s="3"/>
       <c r="F218" s="3"/>
     </row>
-    <row r="219" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="219" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B219" s="3"/>
       <c r="C219" s="3"/>
       <c r="D219" s="3"/>
       <c r="E219" s="3"/>
       <c r="F219" s="3"/>
     </row>
-    <row r="220" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="220" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B220" s="3"/>
       <c r="C220" s="3"/>
       <c r="D220" s="3"/>
       <c r="E220" s="3"/>
       <c r="F220" s="3"/>
     </row>
-    <row r="221" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="221" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B221" s="3"/>
       <c r="C221" s="3"/>
       <c r="D221" s="3"/>
       <c r="E221" s="3"/>
       <c r="F221" s="3"/>
     </row>
-    <row r="222" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="222" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B222" s="3"/>
       <c r="C222" s="3"/>
       <c r="D222" s="3"/>
       <c r="E222" s="3"/>
       <c r="F222" s="3"/>
     </row>
-    <row r="223" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="223" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B223" s="3"/>
       <c r="C223" s="3"/>
       <c r="D223" s="3"/>
       <c r="E223" s="3"/>
       <c r="F223" s="3"/>
     </row>
-    <row r="224" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="224" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B224" s="3"/>
       <c r="C224" s="3"/>
       <c r="D224" s="3"/>
       <c r="E224" s="3"/>
       <c r="F224" s="3"/>
     </row>
-    <row r="225" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="225" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B225" s="3"/>
       <c r="C225" s="3"/>
       <c r="D225" s="3"/>
       <c r="E225" s="3"/>
       <c r="F225" s="3"/>
     </row>
-    <row r="226" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="226" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B226" s="3"/>
       <c r="C226" s="3"/>
       <c r="D226" s="3"/>
       <c r="E226" s="3"/>
       <c r="F226" s="3"/>
     </row>
-    <row r="227" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="227" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B227" s="3"/>
       <c r="C227" s="3"/>
       <c r="D227" s="3"/>
       <c r="E227" s="3"/>
       <c r="F227" s="3"/>
     </row>
-    <row r="228" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="228" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B228" s="3"/>
       <c r="C228" s="3"/>
       <c r="D228" s="3"/>
       <c r="E228" s="3"/>
       <c r="F228" s="3"/>
     </row>
-    <row r="229" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="229" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B229" s="3"/>
       <c r="C229" s="3"/>
       <c r="D229" s="3"/>
       <c r="E229" s="3"/>
       <c r="F229" s="3"/>
     </row>
-    <row r="230" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="230" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B230" s="3"/>
       <c r="C230" s="3"/>
       <c r="D230" s="3"/>
       <c r="E230" s="3"/>
       <c r="F230" s="3"/>
     </row>
-    <row r="231" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="231" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B231" s="3"/>
       <c r="C231" s="3"/>
       <c r="D231" s="3"/>
       <c r="E231" s="3"/>
       <c r="F231" s="3"/>
     </row>
-    <row r="232" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="232" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B232" s="3"/>
       <c r="C232" s="3"/>
       <c r="D232" s="3"/>
       <c r="E232" s="3"/>
       <c r="F232" s="3"/>
     </row>
-    <row r="233" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="233" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B233" s="3"/>
       <c r="C233" s="3"/>
       <c r="D233" s="3"/>
       <c r="E233" s="3"/>
       <c r="F233" s="3"/>
     </row>
-    <row r="234" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="234" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B234" s="3"/>
       <c r="C234" s="3"/>
       <c r="D234" s="3"/>
       <c r="E234" s="3"/>
       <c r="F234" s="3"/>
     </row>
-    <row r="235" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="235" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B235" s="3"/>
       <c r="C235" s="3"/>
       <c r="D235" s="3"/>
       <c r="E235" s="3"/>
       <c r="F235" s="3"/>
     </row>
-    <row r="236" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="236" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B236" s="3"/>
       <c r="C236" s="3"/>
       <c r="D236" s="3"/>
       <c r="E236" s="3"/>
       <c r="F236" s="3"/>
     </row>
-    <row r="237" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="237" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B237" s="3"/>
       <c r="C237" s="3"/>
       <c r="D237" s="3"/>
       <c r="E237" s="3"/>
       <c r="F237" s="3"/>
     </row>
-    <row r="238" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="238" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B238" s="3"/>
       <c r="C238" s="3"/>
       <c r="D238" s="3"/>
       <c r="E238" s="3"/>
       <c r="F238" s="3"/>
     </row>
-    <row r="239" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="239" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B239" s="3"/>
       <c r="C239" s="3"/>
       <c r="D239" s="3"/>
       <c r="E239" s="3"/>
       <c r="F239" s="3"/>
     </row>
-    <row r="240" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="240" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B240" s="3"/>
       <c r="C240" s="3"/>
       <c r="D240" s="3"/>
       <c r="E240" s="3"/>
       <c r="F240" s="3"/>
     </row>
-    <row r="241" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="241" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B241" s="3"/>
       <c r="C241" s="3"/>
       <c r="D241" s="3"/>
       <c r="E241" s="3"/>
       <c r="F241" s="3"/>
     </row>
-    <row r="242" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="242" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B242" s="3"/>
       <c r="C242" s="3"/>
       <c r="D242" s="3"/>
       <c r="E242" s="3"/>
       <c r="F242" s="3"/>
     </row>
-    <row r="243" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="243" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B243" s="3"/>
       <c r="C243" s="3"/>
       <c r="D243" s="3"/>
       <c r="E243" s="3"/>
       <c r="F243" s="3"/>
     </row>
-    <row r="244" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="244" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B244" s="3"/>
       <c r="C244" s="3"/>
       <c r="D244" s="3"/>
       <c r="E244" s="3"/>
       <c r="F244" s="3"/>
     </row>
-    <row r="245" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="245" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B245" s="3"/>
       <c r="C245" s="3"/>
       <c r="D245" s="3"/>
       <c r="E245" s="3"/>
       <c r="F245" s="3"/>
     </row>
-    <row r="246" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="246" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B246" s="3"/>
       <c r="C246" s="3"/>
       <c r="D246" s="3"/>
       <c r="E246" s="3"/>
       <c r="F246" s="3"/>
     </row>
-    <row r="247" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="247" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B247" s="3"/>
       <c r="C247" s="3"/>
       <c r="D247" s="3"/>
       <c r="E247" s="3"/>
       <c r="F247" s="3"/>
     </row>
-    <row r="248" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="248" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B248" s="3"/>
       <c r="C248" s="3"/>
       <c r="D248" s="3"/>
       <c r="E248" s="3"/>
       <c r="F248" s="3"/>
     </row>
-    <row r="249" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="249" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B249" s="3"/>
       <c r="C249" s="3"/>
       <c r="D249" s="3"/>
       <c r="E249" s="3"/>
       <c r="F249" s="3"/>
     </row>
-    <row r="250" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="250" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B250" s="3"/>
       <c r="C250" s="3"/>
       <c r="D250" s="3"/>
       <c r="E250" s="3"/>
       <c r="F250" s="3"/>
     </row>
-    <row r="251" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="251" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B251" s="3"/>
       <c r="C251" s="3"/>
       <c r="D251" s="3"/>
       <c r="E251" s="3"/>
       <c r="F251" s="3"/>
     </row>
-    <row r="252" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="252" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B252" s="3"/>
       <c r="C252" s="3"/>
       <c r="D252" s="3"/>
       <c r="E252" s="3"/>
       <c r="F252" s="3"/>
     </row>
-    <row r="253" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="253" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B253" s="3"/>
       <c r="C253" s="3"/>
       <c r="D253" s="3"/>
       <c r="E253" s="3"/>
       <c r="F253" s="3"/>
     </row>
-    <row r="254" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="254" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B254" s="3"/>
       <c r="C254" s="3"/>
       <c r="D254" s="3"/>
       <c r="E254" s="3"/>
       <c r="F254" s="3"/>
     </row>
-    <row r="255" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="255" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B255" s="3"/>
       <c r="C255" s="3"/>
       <c r="D255" s="3"/>
       <c r="E255" s="3"/>
       <c r="F255" s="3"/>
     </row>
-    <row r="256" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="256" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B256" s="3"/>
       <c r="C256" s="3"/>
       <c r="D256" s="3"/>
       <c r="E256" s="3"/>
       <c r="F256" s="3"/>
     </row>
-    <row r="257" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="257" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B257" s="3"/>
       <c r="C257" s="3"/>
       <c r="D257" s="3"/>
       <c r="E257" s="3"/>
       <c r="F257" s="3"/>
     </row>
-    <row r="258" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="258" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B258" s="3"/>
       <c r="C258" s="3"/>
       <c r="D258" s="3"/>
       <c r="E258" s="3"/>
       <c r="F258" s="3"/>
     </row>
-    <row r="259" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="259" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B259" s="3"/>
       <c r="C259" s="3"/>
       <c r="D259" s="3"/>
       <c r="E259" s="3"/>
       <c r="F259" s="3"/>
     </row>
-    <row r="260" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="260" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B260" s="3"/>
       <c r="C260" s="3"/>
       <c r="D260" s="3"/>
       <c r="E260" s="3"/>
       <c r="F260" s="3"/>
     </row>
-    <row r="261" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="261" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B261" s="3"/>
       <c r="C261" s="3"/>
       <c r="D261" s="3"/>
       <c r="E261" s="3"/>
       <c r="F261" s="3"/>
     </row>
-    <row r="262" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="262" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B262" s="3"/>
       <c r="C262" s="3"/>
       <c r="D262" s="3"/>
       <c r="E262" s="3"/>
       <c r="F262" s="3"/>
     </row>
-    <row r="263" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="263" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B263" s="3"/>
       <c r="C263" s="3"/>
       <c r="D263" s="3"/>
       <c r="E263" s="3"/>
       <c r="F263" s="3"/>
     </row>
-    <row r="264" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="264" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B264" s="3"/>
       <c r="C264" s="3"/>
       <c r="D264" s="3"/>
       <c r="E264" s="3"/>
       <c r="F264" s="3"/>
     </row>
-    <row r="265" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="265" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B265" s="3"/>
       <c r="C265" s="3"/>
       <c r="D265" s="3"/>
       <c r="E265" s="3"/>
       <c r="F265" s="3"/>
     </row>
-    <row r="266" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="266" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B266" s="3"/>
       <c r="C266" s="3"/>
       <c r="D266" s="3"/>
       <c r="E266" s="3"/>
       <c r="F266" s="3"/>
     </row>
-    <row r="267" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="267" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B267" s="3"/>
       <c r="C267" s="3"/>
       <c r="D267" s="3"/>
       <c r="E267" s="3"/>
       <c r="F267" s="3"/>
     </row>
-    <row r="268" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="268" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B268" s="3"/>
       <c r="C268" s="3"/>
       <c r="D268" s="3"/>
       <c r="E268" s="3"/>
       <c r="F268" s="3"/>
     </row>
-    <row r="269" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="269" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B269" s="3"/>
       <c r="C269" s="3"/>
       <c r="D269" s="3"/>
       <c r="E269" s="3"/>
       <c r="F269" s="3"/>
     </row>
-    <row r="270" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="270" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B270" s="3"/>
       <c r="C270" s="3"/>
       <c r="D270" s="3"/>
       <c r="E270" s="3"/>
       <c r="F270" s="3"/>
     </row>
-    <row r="271" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="271" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B271" s="3"/>
       <c r="C271" s="3"/>
       <c r="D271" s="3"/>
       <c r="E271" s="3"/>
       <c r="F271" s="3"/>
     </row>
-    <row r="272" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="272" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B272" s="3"/>
       <c r="C272" s="3"/>
       <c r="D272" s="3"/>
       <c r="E272" s="3"/>
       <c r="F272" s="3"/>
     </row>
-    <row r="273" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="273" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B273" s="3"/>
       <c r="C273" s="3"/>
       <c r="D273" s="3"/>
       <c r="E273" s="3"/>
       <c r="F273" s="3"/>
     </row>
-    <row r="274" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="274" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B274" s="3"/>
       <c r="C274" s="3"/>
       <c r="D274" s="3"/>
       <c r="E274" s="3"/>
       <c r="F274" s="3"/>
     </row>
-    <row r="275" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="275" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B275" s="3"/>
       <c r="C275" s="3"/>
       <c r="D275" s="3"/>
       <c r="E275" s="3"/>
       <c r="F275" s="3"/>
     </row>
-    <row r="276" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="276" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B276" s="3"/>
       <c r="C276" s="3"/>
       <c r="D276" s="3"/>
       <c r="E276" s="3"/>
       <c r="F276" s="3"/>
     </row>
-    <row r="277" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="277" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B277" s="3"/>
       <c r="C277" s="3"/>
       <c r="D277" s="3"/>
       <c r="E277" s="3"/>
       <c r="F277" s="3"/>
     </row>
-    <row r="278" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="278" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B278" s="3"/>
       <c r="C278" s="3"/>
       <c r="D278" s="3"/>
       <c r="E278" s="3"/>
       <c r="F278" s="3"/>
     </row>
-    <row r="279" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="279" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B279" s="3"/>
       <c r="C279" s="3"/>
       <c r="D279" s="3"/>
       <c r="E279" s="3"/>
       <c r="F279" s="3"/>
     </row>
-    <row r="280" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="280" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B280" s="3"/>
       <c r="C280" s="3"/>
       <c r="D280" s="3"/>
       <c r="E280" s="3"/>
       <c r="F280" s="3"/>
     </row>
-    <row r="281" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="281" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B281" s="3"/>
       <c r="C281" s="3"/>
       <c r="D281" s="3"/>
       <c r="E281" s="3"/>
       <c r="F281" s="3"/>
     </row>
-    <row r="282" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="282" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B282" s="3"/>
       <c r="C282" s="3"/>
       <c r="D282" s="3"/>
       <c r="E282" s="3"/>
       <c r="F282" s="3"/>
     </row>
-    <row r="283" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="283" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B283" s="3"/>
       <c r="C283" s="3"/>
       <c r="D283" s="3"/>
       <c r="E283" s="3"/>
       <c r="F283" s="3"/>
     </row>
-    <row r="284" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="284" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B284" s="3"/>
       <c r="C284" s="3"/>
       <c r="D284" s="3"/>
       <c r="E284" s="3"/>
       <c r="F284" s="3"/>
     </row>
-    <row r="285" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="285" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B285" s="3"/>
       <c r="C285" s="3"/>
       <c r="D285" s="3"/>
       <c r="E285" s="3"/>
       <c r="F285" s="3"/>
     </row>
-    <row r="286" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="286" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B286" s="3"/>
       <c r="C286" s="3"/>
       <c r="D286" s="3"/>
       <c r="E286" s="3"/>
       <c r="F286" s="3"/>
     </row>
-    <row r="287" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="287" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B287" s="3"/>
       <c r="C287" s="3"/>
       <c r="D287" s="3"/>
       <c r="E287" s="3"/>
       <c r="F287" s="3"/>
     </row>
-    <row r="288" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="288" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B288" s="3"/>
       <c r="C288" s="3"/>
       <c r="D288" s="3"/>
       <c r="E288" s="3"/>
       <c r="F288" s="3"/>
     </row>
-    <row r="289" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="289" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B289" s="3"/>
       <c r="C289" s="3"/>
       <c r="D289" s="3"/>
       <c r="E289" s="3"/>
       <c r="F289" s="3"/>
     </row>
-    <row r="290" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="290" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B290" s="3"/>
       <c r="C290" s="3"/>
       <c r="D290" s="3"/>
       <c r="E290" s="3"/>
       <c r="F290" s="3"/>
     </row>
-    <row r="291" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="291" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B291" s="3"/>
       <c r="C291" s="3"/>
       <c r="D291" s="3"/>
       <c r="E291" s="3"/>
       <c r="F291" s="3"/>
     </row>
-    <row r="292" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="292" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B292" s="3"/>
       <c r="C292" s="3"/>
       <c r="D292" s="3"/>
       <c r="E292" s="3"/>
       <c r="F292" s="3"/>
     </row>
-    <row r="293" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="293" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B293" s="3"/>
       <c r="C293" s="3"/>
       <c r="D293" s="3"/>
       <c r="E293" s="3"/>
       <c r="F293" s="3"/>
     </row>
-    <row r="294" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="294" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B294" s="3"/>
       <c r="C294" s="3"/>
       <c r="D294" s="3"/>
       <c r="E294" s="3"/>
       <c r="F294" s="3"/>
     </row>
-    <row r="295" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="295" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B295" s="3"/>
       <c r="C295" s="3"/>
       <c r="D295" s="3"/>
       <c r="E295" s="3"/>
       <c r="F295" s="3"/>
     </row>
-    <row r="296" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="296" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B296" s="3"/>
       <c r="C296" s="3"/>
       <c r="D296" s="3"/>
       <c r="E296" s="3"/>
       <c r="F296" s="3"/>
     </row>
-    <row r="297" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="297" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B297" s="3"/>
       <c r="C297" s="3"/>
       <c r="D297" s="3"/>
       <c r="E297" s="3"/>
       <c r="F297" s="3"/>
     </row>
-    <row r="298" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="298" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B298" s="3"/>
       <c r="C298" s="3"/>
       <c r="D298" s="3"/>
       <c r="E298" s="3"/>
       <c r="F298" s="3"/>
     </row>
-    <row r="299" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="299" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B299" s="3"/>
       <c r="C299" s="3"/>
       <c r="D299" s="3"/>
       <c r="E299" s="3"/>
       <c r="F299" s="3"/>
     </row>
-    <row r="300" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="300" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B300" s="3"/>
       <c r="C300" s="3"/>
       <c r="D300" s="3"/>
       <c r="E300" s="3"/>
       <c r="F300" s="3"/>
     </row>
-    <row r="301" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="301" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B301" s="3"/>
       <c r="C301" s="3"/>
       <c r="D301" s="3"/>
       <c r="E301" s="3"/>
       <c r="F301" s="3"/>
     </row>
-    <row r="302" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="302" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B302" s="3"/>
       <c r="C302" s="3"/>
       <c r="D302" s="3"/>
       <c r="E302" s="3"/>
       <c r="F302" s="3"/>
     </row>
-    <row r="303" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="303" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B303" s="3"/>
       <c r="C303" s="3"/>
       <c r="D303" s="3"/>
       <c r="E303" s="3"/>
       <c r="F303" s="3"/>
     </row>
-    <row r="304" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="304" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B304" s="3"/>
       <c r="C304" s="3"/>
       <c r="D304" s="3"/>
       <c r="E304" s="3"/>
       <c r="F304" s="3"/>
     </row>
-    <row r="305" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="305" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B305" s="3"/>
       <c r="C305" s="3"/>
       <c r="D305" s="3"/>
       <c r="E305" s="3"/>
       <c r="F305" s="3"/>
     </row>
-    <row r="306" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="306" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B306" s="3"/>
       <c r="C306" s="3"/>
       <c r="D306" s="3"/>
       <c r="E306" s="3"/>
       <c r="F306" s="3"/>
     </row>
-    <row r="307" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="307" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B307" s="3"/>
       <c r="C307" s="3"/>
       <c r="D307" s="3"/>
       <c r="E307" s="3"/>
       <c r="F307" s="3"/>
     </row>
-    <row r="308" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="308" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B308" s="3"/>
       <c r="C308" s="3"/>
       <c r="D308" s="3"/>
       <c r="E308" s="3"/>
       <c r="F308" s="3"/>
     </row>
-    <row r="309" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="309" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B309" s="3"/>
       <c r="C309" s="3"/>
       <c r="D309" s="3"/>
       <c r="E309" s="3"/>
       <c r="F309" s="3"/>
     </row>
-    <row r="310" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="310" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B310" s="3"/>
       <c r="C310" s="3"/>
       <c r="D310" s="3"/>
       <c r="E310" s="3"/>
       <c r="F310" s="3"/>
     </row>
-    <row r="311" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="311" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B311" s="3"/>
       <c r="C311" s="3"/>
       <c r="D311" s="3"/>
       <c r="E311" s="3"/>
       <c r="F311" s="3"/>
     </row>
-    <row r="312" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="312" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B312" s="3"/>
       <c r="C312" s="3"/>
       <c r="D312" s="3"/>
       <c r="E312" s="3"/>
       <c r="F312" s="3"/>
     </row>
-    <row r="313" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="313" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B313" s="3"/>
       <c r="C313" s="3"/>
       <c r="D313" s="3"/>
       <c r="E313" s="3"/>
       <c r="F313" s="3"/>
     </row>
-    <row r="314" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="314" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B314" s="3"/>
       <c r="C314" s="3"/>
       <c r="D314" s="3"/>
       <c r="E314" s="3"/>
       <c r="F314" s="3"/>
     </row>
-    <row r="315" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="315" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B315" s="3"/>
       <c r="C315" s="3"/>
       <c r="D315" s="3"/>
       <c r="E315" s="3"/>
       <c r="F315" s="3"/>
     </row>
-    <row r="316" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="316" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B316" s="3"/>
       <c r="C316" s="3"/>
       <c r="D316" s="3"/>
       <c r="E316" s="3"/>
       <c r="F316" s="3"/>
     </row>
-    <row r="317" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="317" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B317" s="3"/>
       <c r="C317" s="3"/>
       <c r="D317" s="3"/>
       <c r="E317" s="3"/>
       <c r="F317" s="3"/>
     </row>
-    <row r="318" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="318" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B318" s="3"/>
       <c r="C318" s="3"/>
       <c r="D318" s="3"/>
       <c r="E318" s="3"/>
       <c r="F318" s="3"/>
     </row>
-    <row r="319" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="319" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B319" s="3"/>
       <c r="C319" s="3"/>
       <c r="D319" s="3"/>
       <c r="E319" s="3"/>
       <c r="F319" s="3"/>
     </row>
-    <row r="320" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="320" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B320" s="3"/>
       <c r="C320" s="3"/>
       <c r="D320" s="3"/>
       <c r="E320" s="3"/>
       <c r="F320" s="3"/>
     </row>
-    <row r="321" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="321" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B321" s="3"/>
       <c r="C321" s="3"/>
       <c r="D321" s="3"/>
       <c r="E321" s="3"/>
       <c r="F321" s="3"/>
     </row>
-    <row r="322" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="322" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B322" s="3"/>
       <c r="C322" s="3"/>
       <c r="D322" s="3"/>
       <c r="E322" s="3"/>
       <c r="F322" s="3"/>
     </row>
-    <row r="323" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="323" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B323" s="3"/>
       <c r="C323" s="3"/>
       <c r="D323" s="3"/>
       <c r="E323" s="3"/>
       <c r="F323" s="3"/>
     </row>
-    <row r="324" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="324" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B324" s="3"/>
       <c r="C324" s="3"/>
       <c r="D324" s="3"/>
       <c r="E324" s="3"/>
       <c r="F324" s="3"/>
     </row>
-    <row r="325" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="325" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B325" s="3"/>
       <c r="C325" s="3"/>
       <c r="D325" s="3"/>
       <c r="E325" s="3"/>
       <c r="F325" s="3"/>
     </row>
-    <row r="326" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="326" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B326" s="3"/>
       <c r="C326" s="3"/>
       <c r="D326" s="3"/>
       <c r="E326" s="3"/>
       <c r="F326" s="3"/>
     </row>
-    <row r="327" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="327" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B327" s="3"/>
       <c r="C327" s="3"/>
       <c r="D327" s="3"/>
       <c r="E327" s="3"/>
       <c r="F327" s="3"/>
     </row>
-    <row r="328" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="328" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B328" s="3"/>
       <c r="C328" s="3"/>
       <c r="D328" s="3"/>
       <c r="E328" s="3"/>
       <c r="F328" s="3"/>
     </row>
-    <row r="329" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="329" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B329" s="3"/>
       <c r="C329" s="3"/>
       <c r="D329" s="3"/>
       <c r="E329" s="3"/>
       <c r="F329" s="3"/>
     </row>
-    <row r="330" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="330" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B330" s="3"/>
       <c r="C330" s="3"/>
       <c r="D330" s="3"/>
       <c r="E330" s="3"/>
       <c r="F330" s="3"/>
     </row>
-    <row r="331" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="331" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B331" s="3"/>
       <c r="C331" s="3"/>
       <c r="D331" s="3"/>
       <c r="E331" s="3"/>
       <c r="F331" s="3"/>
     </row>
-    <row r="332" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="332" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B332" s="3"/>
       <c r="C332" s="3"/>
       <c r="D332" s="3"/>
       <c r="E332" s="3"/>
       <c r="F332" s="3"/>
     </row>
-    <row r="333" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="333" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B333" s="3"/>
       <c r="C333" s="3"/>
       <c r="D333" s="3"/>
       <c r="E333" s="3"/>
       <c r="F333" s="3"/>
     </row>
-    <row r="334" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="334" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B334" s="3"/>
       <c r="C334" s="3"/>
       <c r="D334" s="3"/>
       <c r="E334" s="3"/>
       <c r="F334" s="3"/>
     </row>
-    <row r="335" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="335" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B335" s="3"/>
       <c r="C335" s="3"/>
       <c r="D335" s="3"/>
       <c r="E335" s="3"/>
       <c r="F335" s="3"/>
     </row>
+    <row r="336" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B336" s="3"/>
+      <c r="C336" s="3"/>
+      <c r="D336" s="3"/>
+      <c r="E336" s="3"/>
+      <c r="F336" s="3"/>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>